<commit_message>
fix(reports): keep snapshots and exports consistent with canonical data
</commit_message>
<xml_diff>
--- a/docs/qa/reports-01/reports01-filtered.xlsx
+++ b/docs/qa/reports-01/reports01-filtered.xlsx
@@ -97,7 +97,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <v>46313.63313094231</v>
+        <v>46313.665503105425</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -285,7 +285,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Получени доставки (несторнирани)</t>
+          <t xml:space="preserve">Заявки с оставащи позиции</t>
         </is>
       </c>
       <c r="B13" s="0">
@@ -296,48 +296,36 @@
           <t xml:space="preserve">бр.</t>
         </is>
       </c>
-      <c r="D13" s="0">
-        <v>0</v>
-      </c>
-      <c r="E13" s="0">
-        <v>1</v>
-      </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Статистика за периода</t>
+          <t xml:space="preserve">Текущо състояние</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Създадени заявки</t>
+          <t xml:space="preserve">Чака поръчване</t>
         </is>
       </c>
       <c r="B14" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">бр.</t>
         </is>
       </c>
-      <c r="D14" s="0">
-        <v>0</v>
-      </c>
-      <c r="E14" s="0">
-        <v>1</v>
-      </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Статистика за периода</t>
+          <t xml:space="preserve">Текущо състояние</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подадени заявки</t>
+          <t xml:space="preserve">Забавени поръчани заявки</t>
         </is>
       </c>
       <c r="B15" s="0">
@@ -348,22 +336,16 @@
           <t xml:space="preserve">бр.</t>
         </is>
       </c>
-      <c r="D15" s="0">
-        <v>0</v>
-      </c>
-      <c r="E15" s="0">
-        <v>1</v>
-      </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Статистика за периода</t>
+          <t xml:space="preserve">Текущо състояние</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Поръчани заявки</t>
+          <t xml:space="preserve">Получени доставки (несторнирани)</t>
         </is>
       </c>
       <c r="B16" s="0">
@@ -389,7 +371,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Одобрени заявки</t>
+          <t xml:space="preserve">Създадени заявки</t>
         </is>
       </c>
       <c r="B17" s="0">
@@ -415,11 +397,11 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отхвърлени заявки</t>
+          <t xml:space="preserve">Подадени заявки</t>
         </is>
       </c>
       <c r="B18" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -430,7 +412,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
@@ -441,11 +423,11 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отменени заявки</t>
+          <t xml:space="preserve">Поръчани заявки</t>
         </is>
       </c>
       <c r="B19" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -456,7 +438,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="0" t="inlineStr">
         <is>
@@ -467,11 +449,11 @@
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Напълно доставени заявки</t>
+          <t xml:space="preserve">Одобрени заявки</t>
         </is>
       </c>
       <c r="B20" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
@@ -482,7 +464,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
@@ -493,16 +475,22 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Частично доставени (създадени в периода)</t>
+          <t xml:space="preserve">Отхвърлени заявки</t>
         </is>
       </c>
       <c r="B21" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">бр.</t>
         </is>
+      </c>
+      <c r="D21" s="0">
+        <v>0</v>
+      </c>
+      <c r="E21" s="0">
+        <v>0</v>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
@@ -513,51 +501,63 @@
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Незавършени заявки</t>
+          <t xml:space="preserve">Отменени заявки</t>
         </is>
       </c>
       <c r="B22" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">бр.</t>
         </is>
       </c>
+      <c r="D22" s="0">
+        <v>0</v>
+      </c>
+      <c r="E22" s="0">
+        <v>0</v>
+      </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Текущо състояние</t>
+          <t xml:space="preserve">Статистика за периода</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заявки с оставащи позиции</t>
+          <t xml:space="preserve">Напълно доставени заявки</t>
         </is>
       </c>
       <c r="B23" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">бр.</t>
         </is>
       </c>
+      <c r="D23" s="0">
+        <v>0</v>
+      </c>
+      <c r="E23" s="0">
+        <v>0</v>
+      </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Текущо състояние</t>
+          <t xml:space="preserve">Статистика за периода</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чака поръчване</t>
+          <t xml:space="preserve">Частично доставени (създадени в периода)</t>
         </is>
       </c>
       <c r="B24" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -566,45 +566,25 @@
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Текущо състояние</t>
+          <t xml:space="preserve">Статистика за периода</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Забавени поръчани заявки</t>
-        </is>
-      </c>
-      <c r="B25" s="0">
-        <v>1</v>
+          <t xml:space="preserve">Средно време от поръчка до пълна доставка</t>
+        </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">бр.</t>
-        </is>
+          <t xml:space="preserve">ч</t>
+        </is>
+      </c>
+      <c r="G25" s="0">
+        <v>0</v>
       </c>
       <c r="H25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Текущо състояние</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Средно време от поръчка до пълна доставка</t>
-        </is>
-      </c>
-      <c r="C26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ч</t>
-        </is>
-      </c>
-      <c r="G26" s="0">
-        <v>0</v>
-      </c>
-      <c r="H26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Статистика за периода</t>
         </is>
@@ -731,7 +711,7 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <v>46293.632893518516</v>
+        <v>46293.66533564815</v>
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
@@ -755,8 +735,52 @@
         <v>2</v>
       </c>
     </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Получени доставки (несторнирани)</t>
+        </is>
+      </c>
+      <c r="B3" s="0">
+        <v>3</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KK9000</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">№REPORTS-QA-1 Synthetic reports QA 1</t>
+        </is>
+      </c>
+      <c r="E3" s="2">
+        <v>46297.66533564815</v>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Частично доставена</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Synthetic QA request</t>
+        </is>
+      </c>
+      <c r="L3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Synthetic QA item: 4 pcs; Synthetic QA liquid: 5.5 l</t>
+        </is>
+      </c>
+      <c r="M3" s="0">
+        <v>20</v>
+      </c>
+      <c r="N3" s="0">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N2"/>
+  <autoFilter ref="A1:N3"/>
 </worksheet>
 </file>
 
@@ -971,7 +995,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 регистрирани ремонта за последните 14 дни. 1 текущи ремонта над 14 дни. 1 завършени връщания за ремонт за последните 14 дни.</t>
+          <t xml:space="preserve">5 регистрирани ремонта за последните 90 дни. 1 текущи ремонта над 7 дни. 1 завършени връщания за ремонт за последните 90 дни.</t>
         </is>
       </c>
       <c r="C2" s="0">

</xml_diff>

<commit_message>
test(reports): await filtered results before capturing QA evidence
</commit_message>
<xml_diff>
--- a/docs/qa/reports-01/reports01-filtered.xlsx
+++ b/docs/qa/reports-01/reports01-filtered.xlsx
@@ -97,7 +97,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <v>46313.665503105425</v>
+        <v>46313.66912542385</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <v>46293.66533564815</v>
+        <v>46293.66893518518</v>
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="E3" s="2">
-        <v>46297.66533564815</v>
+        <v>46297.66893518518</v>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>

</xml_diff>